<commit_message>
Migrate grace.com/about-grace/ page to Document Authoring
Single-page content migration of the About Grace page, reusing the
existing block library (no new blocks):

- about-grace template added to page-templates.json: full-bleed hero +
  3-column navigation tile grid (8 tiles → About subpages).
- Reuses hero-fullbleed and cards-industry.
- import-about-grace.js orchestrates the shared parsers + transformers,
  and strips the pre-footer Standard Industries logo that otherwise
  leaked into the tile grid.
- cards-industry parser hardened: scope cards to .card-item/.card-group
  and strip the hidden "PROMOTION" eyebrow from tile labels (homepage
  industries grid still validates 100%).

Content uploaded to DA and published; renders at /about-grace/.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-products.report.xlsx
+++ b/tools/importer/reports/import-products.report.xlsx
@@ -64,13 +64,13 @@
     <t>products.report.json</t>
   </si>
   <si>
-    <t>["hero-fullbleed","hero-fullbleed","cards-product","cards-product","cards-insights","cards-insights"]</t>
+    <t>["hero-fullbleed","hero-fullbleed","cards-product","cards-product","cards-insights"]</t>
   </si>
   <si>
     <t>products</t>
   </si>
   <si>
-    <t>2026-08-26T20:12:47.932Z</t>
+    <t>2026-08-26T20:35:34.948Z</t>
   </si>
   <si>
     <t>Products</t>

</xml_diff>